<commit_message>
data(layout): 24 ubicaciones nuevas contra el rack agregado en el v3 (384 en total)
Se generan con la misma logica deducida de las demas: pick_sequence en zigzag
por columna (indice 15, descendente 384..361), area en bloques de 2 filas sin
repetir el bloque anterior, WorkGroup atado al area (A/B/C) y SKU/cantidad del
mismo rango. Reparto final: 154 Ground, 154 High, 76 Special.

Medido con la estacion activa y semilla 42: 4+4 repartido 4.450 s,
8+8 repartido 2.574 s, 4+4 todo al carril 1 8.682 s.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/layouts/Warehouse_Logic_v3.xlsx
+++ b/layouts/Warehouse_Logic_v3.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G361"/>
+  <dimension ref="A1:G385"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="3" bestFit="1" customWidth="1" min="1" max="2"/>
@@ -10923,6 +10923,702 @@
       <c r="G361" t="inlineStr">
         <is>
           <t>Area_Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>30</v>
+      </c>
+      <c r="B362" t="n">
+        <v>3</v>
+      </c>
+      <c r="C362" t="n">
+        <v>384</v>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>SKU039</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>37</v>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>30</v>
+      </c>
+      <c r="B363" t="n">
+        <v>4</v>
+      </c>
+      <c r="C363" t="n">
+        <v>383</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>SKU017</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>26</v>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>30</v>
+      </c>
+      <c r="B364" t="n">
+        <v>5</v>
+      </c>
+      <c r="C364" t="n">
+        <v>382</v>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>SKU042</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>81</v>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>30</v>
+      </c>
+      <c r="B365" t="n">
+        <v>6</v>
+      </c>
+      <c r="C365" t="n">
+        <v>381</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>SKU024</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>90</v>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>30</v>
+      </c>
+      <c r="B366" t="n">
+        <v>7</v>
+      </c>
+      <c r="C366" t="n">
+        <v>380</v>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>SKU007</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>86</v>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>30</v>
+      </c>
+      <c r="B367" t="n">
+        <v>8</v>
+      </c>
+      <c r="C367" t="n">
+        <v>379</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>SKU008</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>56</v>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>30</v>
+      </c>
+      <c r="B368" t="n">
+        <v>9</v>
+      </c>
+      <c r="C368" t="n">
+        <v>378</v>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>SKU006</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>40</v>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>WG_C</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Area_Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>30</v>
+      </c>
+      <c r="B369" t="n">
+        <v>10</v>
+      </c>
+      <c r="C369" t="n">
+        <v>377</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>SKU018</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>77</v>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>WG_C</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Area_Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>30</v>
+      </c>
+      <c r="B370" t="n">
+        <v>11</v>
+      </c>
+      <c r="C370" t="n">
+        <v>376</v>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>SKU033</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>38</v>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>30</v>
+      </c>
+      <c r="B371" t="n">
+        <v>12</v>
+      </c>
+      <c r="C371" t="n">
+        <v>375</v>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>SKU028</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>31</v>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>30</v>
+      </c>
+      <c r="B372" t="n">
+        <v>13</v>
+      </c>
+      <c r="C372" t="n">
+        <v>374</v>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>SKU015</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>77</v>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>30</v>
+      </c>
+      <c r="B373" t="n">
+        <v>14</v>
+      </c>
+      <c r="C373" t="n">
+        <v>373</v>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>SKU023</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>23</v>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>30</v>
+      </c>
+      <c r="B374" t="n">
+        <v>15</v>
+      </c>
+      <c r="C374" t="n">
+        <v>372</v>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>SKU027</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>26</v>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>30</v>
+      </c>
+      <c r="B375" t="n">
+        <v>16</v>
+      </c>
+      <c r="C375" t="n">
+        <v>371</v>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>SKU026</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>84</v>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>30</v>
+      </c>
+      <c r="B376" t="n">
+        <v>17</v>
+      </c>
+      <c r="C376" t="n">
+        <v>370</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>SKU024</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>50</v>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>WG_C</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Area_Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>30</v>
+      </c>
+      <c r="B377" t="n">
+        <v>18</v>
+      </c>
+      <c r="C377" t="n">
+        <v>369</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>SKU025</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>30</v>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>WG_C</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Area_Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>30</v>
+      </c>
+      <c r="B378" t="n">
+        <v>19</v>
+      </c>
+      <c r="C378" t="n">
+        <v>368</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>SKU024</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>48</v>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>30</v>
+      </c>
+      <c r="B379" t="n">
+        <v>20</v>
+      </c>
+      <c r="C379" t="n">
+        <v>367</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>SKU002</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>60</v>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>30</v>
+      </c>
+      <c r="B380" t="n">
+        <v>21</v>
+      </c>
+      <c r="C380" t="n">
+        <v>366</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>SKU007</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>62</v>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>30</v>
+      </c>
+      <c r="B381" t="n">
+        <v>22</v>
+      </c>
+      <c r="C381" t="n">
+        <v>365</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>SKU010</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>37</v>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>30</v>
+      </c>
+      <c r="B382" t="n">
+        <v>23</v>
+      </c>
+      <c r="C382" t="n">
+        <v>364</v>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>SKU003</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>56</v>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>30</v>
+      </c>
+      <c r="B383" t="n">
+        <v>24</v>
+      </c>
+      <c r="C383" t="n">
+        <v>363</v>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>SKU031</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>37</v>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>WG_B</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Area_High</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>30</v>
+      </c>
+      <c r="B384" t="n">
+        <v>25</v>
+      </c>
+      <c r="C384" t="n">
+        <v>362</v>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>SKU049</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>80</v>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>30</v>
+      </c>
+      <c r="B385" t="n">
+        <v>26</v>
+      </c>
+      <c r="C385" t="n">
+        <v>361</v>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>SKU029</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>98</v>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>WG_A</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Area_Ground</t>
         </is>
       </c>
     </row>

</xml_diff>